<commit_message>
fix: bump workbook SCHEMA_VERSION to 2 for the user-email attribution columns (#2278)
Version-1 workbooks hold raw user uuids in entered_by, submitted_by,
overridden_by, committed_by, approved_by and created_by. Since #2278 those
columns resolve against the users tab by email, so every such row in an old
file became a row error. meta.ts says the version is bumped when a change makes
an older workbook unreadable, so it is now 2 and readWorkbook refuses a v1 file
up front with UNSUPPORTED_VERSION ("This workbook uses schema version 1 ...").
Pre-launch, so no v1 migration path is kept. The checked-in .xlsx fixtures are
regenerated with make-fixtures.ts.

Review of PR #2422, finding 3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/test/fixtures/workbook/three-errors.xlsx
+++ b/server/test/fixtures/workbook/three-errors.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
   <si>
     <t>key</t>
   </si>
@@ -72,6 +72,9 @@
   </si>
   <si>
     <t>registration_id</t>
+  </si>
+  <si>
+    <t>country_code</t>
   </si>
   <si>
     <t>settings</t>
@@ -482,7 +485,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -533,10 +536,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -561,83 +564,86 @@
       <c r="H1" t="s">
         <v>20</v>
       </c>
+      <c r="I1" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>